<commit_message>
Préparation pour les experts et complétion de l'implémentation
</commit_message>
<xml_diff>
--- a/Doc/3_CAND_Modele_Journal_2026.xlsx
+++ b/Doc/3_CAND_Modele_Journal_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TPI - 2026 - Lucielle Voeffray\Dossier de projet\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47308637-90E4-49D1-99C9-9B058518078D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCF1A169-8DE8-4FA7-AF96-7E2163A72C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="8" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="22">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
   </si>
@@ -130,6 +130,15 @@
   </si>
   <si>
     <t>D'habitude l'analyse me fait des soucis, visiblement les derniers modules ont bien permis de m'habituer à celle-ci.</t>
+  </si>
+  <si>
+    <t>Préparation au rendez-vous expert</t>
+  </si>
+  <si>
+    <t>DOC - Exigences techniques et fonctionnelles</t>
+  </si>
+  <si>
+    <t>DOC - Concept d'implémentation</t>
   </si>
 </sst>
 </file>
@@ -483,108 +492,108 @@
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
@@ -1228,107 +1237,107 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
     </row>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="38" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="37"/>
+      <c r="B2" s="38"/>
+      <c r="C2" s="39"/>
       <c r="D2" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="32" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="B4" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="31"/>
+      <c r="C4" s="33"/>
       <c r="D4" s="5" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="32"/>
-      <c r="B5" s="32"/>
-      <c r="C5" s="33"/>
+      <c r="A5" s="34"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="35"/>
       <c r="D5" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="38">
+      <c r="A6" s="28">
         <v>46153</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="36" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="35"/>
+      <c r="C6" s="37"/>
       <c r="D6" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="17"/>
-      <c r="B7" s="20" t="s">
+      <c r="A7" s="16"/>
+      <c r="B7" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="21"/>
+      <c r="C7" s="20"/>
       <c r="D7" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="17"/>
-      <c r="B8" s="20" t="s">
+      <c r="A8" s="16"/>
+      <c r="B8" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="21"/>
+      <c r="C8" s="20"/>
       <c r="D8" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="17"/>
-      <c r="B9" s="20" t="s">
+      <c r="A9" s="16"/>
+      <c r="B9" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="21"/>
+      <c r="C9" s="20"/>
       <c r="D9" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="17"/>
-      <c r="B10" s="20" t="s">
+      <c r="A10" s="16"/>
+      <c r="B10" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="21"/>
+      <c r="C10" s="20"/>
       <c r="D10" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="17"/>
-      <c r="B11" s="20" t="s">
+      <c r="A11" s="16"/>
+      <c r="B11" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="21"/>
+      <c r="C11" s="20"/>
       <c r="D11" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="17"/>
+      <c r="A12" s="16"/>
       <c r="B12" s="13" t="s">
         <v>16</v>
       </c>
@@ -1338,13 +1347,13 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="17"/>
-      <c r="B13" s="39"/>
-      <c r="C13" s="40"/>
+      <c r="A13" s="16"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="30"/>
       <c r="D13" s="8"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="17"/>
+      <c r="A14" s="16"/>
       <c r="B14" s="2" t="s">
         <v>8</v>
       </c>
@@ -1357,47 +1366,59 @@
       </c>
     </row>
     <row r="15" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="17"/>
-      <c r="B15" s="22" t="s">
+      <c r="A15" s="16"/>
+      <c r="B15" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="C15" s="23"/>
-      <c r="D15" s="24"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="23"/>
     </row>
     <row r="16" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="16">
+      <c r="A16" s="15">
         <v>46154</v>
       </c>
-      <c r="B16" s="18"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="7"/>
+      <c r="B16" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C16" s="18"/>
+      <c r="D16" s="7">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="17"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="8"/>
+      <c r="A17" s="16"/>
+      <c r="B17" s="19" t="s">
+        <v>20</v>
+      </c>
+      <c r="C17" s="20"/>
+      <c r="D17" s="8">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="17"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="8"/>
+      <c r="A18" s="16"/>
+      <c r="B18" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C18" s="20"/>
+      <c r="D18" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="17"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="21"/>
+      <c r="A19" s="16"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="20"/>
       <c r="D19" s="8"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="17"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="21"/>
+      <c r="A20" s="16"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="20"/>
       <c r="D20" s="8"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="17"/>
+      <c r="A21" s="16"/>
       <c r="B21" s="2" t="s">
         <v>8</v>
       </c>
@@ -1406,47 +1427,47 @@
       </c>
       <c r="D21" s="9">
         <f>SUM(D16:D20)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="17"/>
-      <c r="B22" s="22"/>
-      <c r="C22" s="23"/>
-      <c r="D22" s="24"/>
+      <c r="A22" s="16"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="23"/>
     </row>
     <row r="23" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="16"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="19"/>
+      <c r="A23" s="15"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="18"/>
       <c r="D23" s="7"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="17"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="21"/>
+      <c r="A24" s="16"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="20"/>
       <c r="D24" s="8"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="17"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="21"/>
+      <c r="A25" s="16"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="20"/>
       <c r="D25" s="8"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="17"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="21"/>
+      <c r="A26" s="16"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="20"/>
       <c r="D26" s="8"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="17"/>
-      <c r="B27" s="20"/>
-      <c r="C27" s="21"/>
+      <c r="A27" s="16"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="20"/>
       <c r="D27" s="8"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="17"/>
+      <c r="A28" s="16"/>
       <c r="B28" s="2" t="s">
         <v>8</v>
       </c>
@@ -1459,43 +1480,43 @@
       </c>
     </row>
     <row r="29" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="17"/>
-      <c r="B29" s="22"/>
-      <c r="C29" s="23"/>
-      <c r="D29" s="24"/>
+      <c r="A29" s="16"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="23"/>
     </row>
     <row r="30" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="16"/>
-      <c r="B30" s="18"/>
-      <c r="C30" s="19"/>
+      <c r="A30" s="15"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="18"/>
       <c r="D30" s="7"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="17"/>
-      <c r="B31" s="20"/>
-      <c r="C31" s="21"/>
+      <c r="A31" s="16"/>
+      <c r="B31" s="19"/>
+      <c r="C31" s="20"/>
       <c r="D31" s="8"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="17"/>
-      <c r="B32" s="20"/>
-      <c r="C32" s="21"/>
+      <c r="A32" s="16"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="20"/>
       <c r="D32" s="8"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="17"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="21"/>
+      <c r="A33" s="16"/>
+      <c r="B33" s="19"/>
+      <c r="C33" s="20"/>
       <c r="D33" s="8"/>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="17"/>
-      <c r="B34" s="20"/>
-      <c r="C34" s="21"/>
+      <c r="A34" s="16"/>
+      <c r="B34" s="19"/>
+      <c r="C34" s="20"/>
       <c r="D34" s="8"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="17"/>
+      <c r="A35" s="16"/>
       <c r="B35" s="2" t="s">
         <v>8</v>
       </c>
@@ -1508,43 +1529,43 @@
       </c>
     </row>
     <row r="36" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="25"/>
-      <c r="B36" s="26"/>
-      <c r="C36" s="27"/>
-      <c r="D36" s="28"/>
+      <c r="A36" s="27"/>
+      <c r="B36" s="24"/>
+      <c r="C36" s="25"/>
+      <c r="D36" s="26"/>
     </row>
     <row r="37" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="16"/>
-      <c r="B37" s="18"/>
-      <c r="C37" s="19"/>
+      <c r="A37" s="15"/>
+      <c r="B37" s="17"/>
+      <c r="C37" s="18"/>
       <c r="D37" s="7"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="17"/>
-      <c r="B38" s="20"/>
-      <c r="C38" s="21"/>
+      <c r="A38" s="16"/>
+      <c r="B38" s="19"/>
+      <c r="C38" s="20"/>
       <c r="D38" s="8"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="17"/>
-      <c r="B39" s="20"/>
-      <c r="C39" s="21"/>
+      <c r="A39" s="16"/>
+      <c r="B39" s="19"/>
+      <c r="C39" s="20"/>
       <c r="D39" s="8"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A40" s="17"/>
-      <c r="B40" s="20"/>
-      <c r="C40" s="21"/>
+      <c r="A40" s="16"/>
+      <c r="B40" s="19"/>
+      <c r="C40" s="20"/>
       <c r="D40" s="8"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A41" s="17"/>
-      <c r="B41" s="20"/>
-      <c r="C41" s="21"/>
+      <c r="A41" s="16"/>
+      <c r="B41" s="19"/>
+      <c r="C41" s="20"/>
       <c r="D41" s="8"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="17"/>
+      <c r="A42" s="16"/>
       <c r="B42" s="2" t="s">
         <v>8</v>
       </c>
@@ -1557,43 +1578,43 @@
       </c>
     </row>
     <row r="43" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="25"/>
-      <c r="B43" s="26"/>
-      <c r="C43" s="27"/>
-      <c r="D43" s="28"/>
+      <c r="A43" s="27"/>
+      <c r="B43" s="24"/>
+      <c r="C43" s="25"/>
+      <c r="D43" s="26"/>
     </row>
     <row r="44" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="16"/>
-      <c r="B44" s="18"/>
-      <c r="C44" s="19"/>
+      <c r="A44" s="15"/>
+      <c r="B44" s="17"/>
+      <c r="C44" s="18"/>
       <c r="D44" s="7"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="17"/>
-      <c r="B45" s="20"/>
-      <c r="C45" s="21"/>
+      <c r="A45" s="16"/>
+      <c r="B45" s="19"/>
+      <c r="C45" s="20"/>
       <c r="D45" s="8"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="17"/>
-      <c r="B46" s="20"/>
-      <c r="C46" s="21"/>
+      <c r="A46" s="16"/>
+      <c r="B46" s="19"/>
+      <c r="C46" s="20"/>
       <c r="D46" s="8"/>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="17"/>
-      <c r="B47" s="20"/>
-      <c r="C47" s="21"/>
+      <c r="A47" s="16"/>
+      <c r="B47" s="19"/>
+      <c r="C47" s="20"/>
       <c r="D47" s="8"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="17"/>
-      <c r="B48" s="20"/>
-      <c r="C48" s="21"/>
+      <c r="A48" s="16"/>
+      <c r="B48" s="19"/>
+      <c r="C48" s="20"/>
       <c r="D48" s="8"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="17"/>
+      <c r="A49" s="16"/>
       <c r="B49" s="2" t="s">
         <v>8</v>
       </c>
@@ -1606,43 +1627,43 @@
       </c>
     </row>
     <row r="50" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="25"/>
-      <c r="B50" s="26"/>
-      <c r="C50" s="27"/>
-      <c r="D50" s="28"/>
+      <c r="A50" s="27"/>
+      <c r="B50" s="24"/>
+      <c r="C50" s="25"/>
+      <c r="D50" s="26"/>
     </row>
     <row r="51" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="16"/>
-      <c r="B51" s="18"/>
-      <c r="C51" s="19"/>
+      <c r="A51" s="15"/>
+      <c r="B51" s="17"/>
+      <c r="C51" s="18"/>
       <c r="D51" s="7"/>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A52" s="17"/>
-      <c r="B52" s="20"/>
-      <c r="C52" s="21"/>
+      <c r="A52" s="16"/>
+      <c r="B52" s="19"/>
+      <c r="C52" s="20"/>
       <c r="D52" s="8"/>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="17"/>
-      <c r="B53" s="20"/>
-      <c r="C53" s="21"/>
+      <c r="A53" s="16"/>
+      <c r="B53" s="19"/>
+      <c r="C53" s="20"/>
       <c r="D53" s="8"/>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="17"/>
-      <c r="B54" s="20"/>
-      <c r="C54" s="21"/>
+      <c r="A54" s="16"/>
+      <c r="B54" s="19"/>
+      <c r="C54" s="20"/>
       <c r="D54" s="8"/>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="17"/>
-      <c r="B55" s="20"/>
-      <c r="C55" s="21"/>
+      <c r="A55" s="16"/>
+      <c r="B55" s="19"/>
+      <c r="C55" s="20"/>
       <c r="D55" s="8"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="17"/>
+      <c r="A56" s="16"/>
       <c r="B56" s="2" t="s">
         <v>8</v>
       </c>
@@ -1655,43 +1676,43 @@
       </c>
     </row>
     <row r="57" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="25"/>
-      <c r="B57" s="26"/>
-      <c r="C57" s="27"/>
-      <c r="D57" s="28"/>
+      <c r="A57" s="27"/>
+      <c r="B57" s="24"/>
+      <c r="C57" s="25"/>
+      <c r="D57" s="26"/>
     </row>
     <row r="58" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="16"/>
-      <c r="B58" s="18"/>
-      <c r="C58" s="19"/>
+      <c r="A58" s="15"/>
+      <c r="B58" s="17"/>
+      <c r="C58" s="18"/>
       <c r="D58" s="7"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A59" s="17"/>
-      <c r="B59" s="20"/>
-      <c r="C59" s="21"/>
+      <c r="A59" s="16"/>
+      <c r="B59" s="19"/>
+      <c r="C59" s="20"/>
       <c r="D59" s="8"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="17"/>
-      <c r="B60" s="20"/>
-      <c r="C60" s="21"/>
+      <c r="A60" s="16"/>
+      <c r="B60" s="19"/>
+      <c r="C60" s="20"/>
       <c r="D60" s="8"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="17"/>
-      <c r="B61" s="20"/>
-      <c r="C61" s="21"/>
+      <c r="A61" s="16"/>
+      <c r="B61" s="19"/>
+      <c r="C61" s="20"/>
       <c r="D61" s="8"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="17"/>
-      <c r="B62" s="20"/>
-      <c r="C62" s="21"/>
+      <c r="A62" s="16"/>
+      <c r="B62" s="19"/>
+      <c r="C62" s="20"/>
       <c r="D62" s="8"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="17"/>
+      <c r="A63" s="16"/>
       <c r="B63" s="2" t="s">
         <v>8</v>
       </c>
@@ -1704,43 +1725,43 @@
       </c>
     </row>
     <row r="64" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="25"/>
-      <c r="B64" s="26"/>
-      <c r="C64" s="27"/>
-      <c r="D64" s="28"/>
+      <c r="A64" s="27"/>
+      <c r="B64" s="24"/>
+      <c r="C64" s="25"/>
+      <c r="D64" s="26"/>
     </row>
     <row r="65" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="16"/>
-      <c r="B65" s="18"/>
-      <c r="C65" s="19"/>
+      <c r="A65" s="15"/>
+      <c r="B65" s="17"/>
+      <c r="C65" s="18"/>
       <c r="D65" s="7"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A66" s="17"/>
-      <c r="B66" s="20"/>
-      <c r="C66" s="21"/>
+      <c r="A66" s="16"/>
+      <c r="B66" s="19"/>
+      <c r="C66" s="20"/>
       <c r="D66" s="8"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="17"/>
-      <c r="B67" s="20"/>
-      <c r="C67" s="21"/>
+      <c r="A67" s="16"/>
+      <c r="B67" s="19"/>
+      <c r="C67" s="20"/>
       <c r="D67" s="8"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="17"/>
-      <c r="B68" s="20"/>
-      <c r="C68" s="21"/>
+      <c r="A68" s="16"/>
+      <c r="B68" s="19"/>
+      <c r="C68" s="20"/>
       <c r="D68" s="8"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="17"/>
-      <c r="B69" s="20"/>
-      <c r="C69" s="21"/>
+      <c r="A69" s="16"/>
+      <c r="B69" s="19"/>
+      <c r="C69" s="20"/>
       <c r="D69" s="8"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="17"/>
+      <c r="A70" s="16"/>
       <c r="B70" s="2" t="s">
         <v>8</v>
       </c>
@@ -1753,43 +1774,43 @@
       </c>
     </row>
     <row r="71" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="17"/>
-      <c r="B71" s="22"/>
-      <c r="C71" s="23"/>
-      <c r="D71" s="24"/>
+      <c r="A71" s="16"/>
+      <c r="B71" s="21"/>
+      <c r="C71" s="22"/>
+      <c r="D71" s="23"/>
     </row>
     <row r="72" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="16"/>
-      <c r="B72" s="18"/>
-      <c r="C72" s="19"/>
+      <c r="A72" s="15"/>
+      <c r="B72" s="17"/>
+      <c r="C72" s="18"/>
       <c r="D72" s="7"/>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A73" s="17"/>
-      <c r="B73" s="20"/>
-      <c r="C73" s="21"/>
+      <c r="A73" s="16"/>
+      <c r="B73" s="19"/>
+      <c r="C73" s="20"/>
       <c r="D73" s="8"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="17"/>
-      <c r="B74" s="20"/>
-      <c r="C74" s="21"/>
+      <c r="A74" s="16"/>
+      <c r="B74" s="19"/>
+      <c r="C74" s="20"/>
       <c r="D74" s="8"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="17"/>
-      <c r="B75" s="20"/>
-      <c r="C75" s="21"/>
+      <c r="A75" s="16"/>
+      <c r="B75" s="19"/>
+      <c r="C75" s="20"/>
       <c r="D75" s="8"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="17"/>
-      <c r="B76" s="20"/>
-      <c r="C76" s="21"/>
+      <c r="A76" s="16"/>
+      <c r="B76" s="19"/>
+      <c r="C76" s="20"/>
       <c r="D76" s="8"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="17"/>
+      <c r="A77" s="16"/>
       <c r="B77" s="2" t="s">
         <v>8</v>
       </c>
@@ -1802,43 +1823,43 @@
       </c>
     </row>
     <row r="78" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="25"/>
-      <c r="B78" s="26"/>
-      <c r="C78" s="27"/>
-      <c r="D78" s="28"/>
+      <c r="A78" s="27"/>
+      <c r="B78" s="24"/>
+      <c r="C78" s="25"/>
+      <c r="D78" s="26"/>
     </row>
     <row r="79" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="16"/>
-      <c r="B79" s="18"/>
-      <c r="C79" s="19"/>
+      <c r="A79" s="15"/>
+      <c r="B79" s="17"/>
+      <c r="C79" s="18"/>
       <c r="D79" s="7"/>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A80" s="17"/>
-      <c r="B80" s="20"/>
-      <c r="C80" s="21"/>
+      <c r="A80" s="16"/>
+      <c r="B80" s="19"/>
+      <c r="C80" s="20"/>
       <c r="D80" s="8"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="17"/>
-      <c r="B81" s="20"/>
-      <c r="C81" s="21"/>
+      <c r="A81" s="16"/>
+      <c r="B81" s="19"/>
+      <c r="C81" s="20"/>
       <c r="D81" s="8"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="17"/>
-      <c r="B82" s="20"/>
-      <c r="C82" s="21"/>
+      <c r="A82" s="16"/>
+      <c r="B82" s="19"/>
+      <c r="C82" s="20"/>
       <c r="D82" s="8"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="17"/>
-      <c r="B83" s="20"/>
-      <c r="C83" s="21"/>
+      <c r="A83" s="16"/>
+      <c r="B83" s="19"/>
+      <c r="C83" s="20"/>
       <c r="D83" s="8"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="17"/>
+      <c r="A84" s="16"/>
       <c r="B84" s="2" t="s">
         <v>8</v>
       </c>
@@ -1851,10 +1872,10 @@
       </c>
     </row>
     <row r="85" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="25"/>
-      <c r="B85" s="26"/>
-      <c r="C85" s="27"/>
-      <c r="D85" s="28"/>
+      <c r="A85" s="27"/>
+      <c r="B85" s="24"/>
+      <c r="C85" s="25"/>
+      <c r="D85" s="26"/>
     </row>
     <row r="86" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="11"/>
@@ -1864,53 +1885,53 @@
       </c>
       <c r="D86" s="12">
         <f>D14+D21+D28+D35+D42+D49+D56+D63+D70+D77+D84</f>
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A87" s="15" t="s">
+      <c r="A87" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B87" s="15"/>
-      <c r="C87" s="15"/>
-      <c r="D87" s="15"/>
+      <c r="B87" s="40"/>
+      <c r="C87" s="40"/>
+      <c r="D87" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="84">
-    <mergeCell ref="A23:A29"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B29:D29"/>
-    <mergeCell ref="B57:D57"/>
-    <mergeCell ref="A58:A64"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="B60:C60"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B62:C62"/>
-    <mergeCell ref="B64:D64"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="A79:A85"/>
-    <mergeCell ref="B79:C79"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="B81:C81"/>
-    <mergeCell ref="B82:C82"/>
-    <mergeCell ref="B83:C83"/>
-    <mergeCell ref="B85:D85"/>
-    <mergeCell ref="A72:A78"/>
-    <mergeCell ref="B72:C72"/>
-    <mergeCell ref="B73:C73"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B75:C75"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B78:D78"/>
+    <mergeCell ref="A87:D87"/>
+    <mergeCell ref="A16:A22"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="A30:A36"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="A37:A43"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="A6:A15"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B41:C41"/>
     <mergeCell ref="B43:D43"/>
     <mergeCell ref="A65:A71"/>
     <mergeCell ref="B65:C65"/>
@@ -1927,40 +1948,40 @@
     <mergeCell ref="B48:C48"/>
     <mergeCell ref="B50:D50"/>
     <mergeCell ref="A51:A57"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="A6:A15"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B4:C5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="A87:D87"/>
-    <mergeCell ref="A16:A22"/>
-    <mergeCell ref="B16:C16"/>
-    <mergeCell ref="B17:C17"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B22:D22"/>
-    <mergeCell ref="A30:A36"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B36:D36"/>
-    <mergeCell ref="A37:A43"/>
+    <mergeCell ref="A72:A78"/>
+    <mergeCell ref="B72:C72"/>
+    <mergeCell ref="B73:C73"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B75:C75"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B78:D78"/>
+    <mergeCell ref="A79:A85"/>
+    <mergeCell ref="B79:C79"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B81:C81"/>
+    <mergeCell ref="B82:C82"/>
+    <mergeCell ref="B83:C83"/>
+    <mergeCell ref="B85:D85"/>
+    <mergeCell ref="B51:C51"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="B57:D57"/>
+    <mergeCell ref="A58:A64"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="B60:C60"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B62:C62"/>
+    <mergeCell ref="B64:D64"/>
+    <mergeCell ref="A23:A29"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B29:D29"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:D14">
     <cfRule type="containsText" dxfId="23" priority="23" operator="containsText" text="Terminé">

</xml_diff>

<commit_message>
FIn de la journée
</commit_message>
<xml_diff>
--- a/Doc/3_CAND_Modele_Journal_2026.xlsx
+++ b/Doc/3_CAND_Modele_Journal_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TPI - 2026 - Lucielle Voeffray\Dossier de projet\Doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13FA3DEA-F154-4E34-ACD1-D5DBE779A33A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27647D7A-972C-4EF1-8A37-5718DC958C5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="48">
   <si>
     <t>Insérer les lignes au-dessus de celle-ci !</t>
   </si>
@@ -205,6 +205,43 @@
   <si>
     <t>Créer Template</t>
   </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Playbook qui reçoit un 403: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF92D050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Problème et solution au point 6.2.4</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Playbook ne trouve pas le template: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="8"/>
+        <color rgb="FF92D050"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Problème et solution au point 6.2.3</t>
+    </r>
+  </si>
+  <si>
+    <t>J'ai passé 2h sur une erreur d'orthographe T-T Vraiment je me fatigue</t>
+  </si>
+  <si>
+    <t>Créer le playbook pour créer les VMs</t>
+  </si>
+  <si>
+    <t>Créer le playbook pour détruire les VMs</t>
+  </si>
 </sst>
 </file>
 
@@ -214,7 +251,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yy;@"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -280,6 +317,12 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color rgb="FF92D050"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -484,7 +527,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
@@ -533,6 +576,74 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0"/>
@@ -542,66 +653,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -654,14 +705,6 @@
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -675,21 +718,57 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="24">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -1282,129 +1361,129 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="20.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="33" t="s">
+      <c r="A1" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
     </row>
     <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="38"/>
-      <c r="C2" s="39"/>
+      <c r="B2" s="40"/>
+      <c r="C2" s="41"/>
       <c r="D2" s="4">
         <v>157443</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="34" t="s">
+      <c r="A4" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="34" t="s">
+      <c r="B4" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="35"/>
+      <c r="C4" s="37"/>
       <c r="D4" s="5" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="36"/>
-      <c r="B5" s="36"/>
-      <c r="C5" s="37"/>
+      <c r="A5" s="38"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="39"/>
       <c r="D5" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="40">
+      <c r="A6" s="42">
         <v>46153</v>
       </c>
-      <c r="B6" s="17" t="s">
+      <c r="B6" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="18"/>
+      <c r="C6" s="16"/>
       <c r="D6" s="7">
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="21"/>
-      <c r="B7" s="17" t="s">
+      <c r="A7" s="23"/>
+      <c r="B7" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="18"/>
+      <c r="C7" s="16"/>
       <c r="D7" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="21"/>
-      <c r="B8" s="17" t="s">
+      <c r="A8" s="23"/>
+      <c r="B8" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="18"/>
+      <c r="C8" s="16"/>
       <c r="D8" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="21"/>
-      <c r="B9" s="17" t="s">
+      <c r="A9" s="23"/>
+      <c r="B9" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C9" s="18"/>
+      <c r="C9" s="16"/>
       <c r="D9" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="21"/>
-      <c r="B10" s="17" t="s">
+      <c r="A10" s="23"/>
+      <c r="B10" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C10" s="18"/>
+      <c r="C10" s="16"/>
       <c r="D10" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="21"/>
-      <c r="B11" s="17" t="s">
+      <c r="A11" s="23"/>
+      <c r="B11" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="18"/>
+      <c r="C11" s="16"/>
       <c r="D11" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="21"/>
-      <c r="B12" s="17" t="s">
+      <c r="A12" s="23"/>
+      <c r="B12" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="18"/>
+      <c r="C12" s="16"/>
       <c r="D12" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="21"/>
-      <c r="B13" s="17"/>
-      <c r="C13" s="18"/>
+      <c r="A13" s="23"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="16"/>
       <c r="D13" s="8"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="21"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="16"/>
+      <c r="A14" s="23"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="14"/>
       <c r="D14" s="8"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="21"/>
+      <c r="A15" s="23"/>
       <c r="B15" s="2" t="s">
         <v>6</v>
       </c>
@@ -1417,74 +1496,74 @@
       </c>
     </row>
     <row r="16" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="21"/>
-      <c r="B16" s="22" t="s">
+      <c r="A16" s="23"/>
+      <c r="B16" s="24" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="23"/>
-      <c r="D16" s="24"/>
+      <c r="C16" s="25"/>
+      <c r="D16" s="26"/>
     </row>
     <row r="17" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="20">
+      <c r="A17" s="22">
         <v>46154</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B17" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C17" s="18"/>
+      <c r="C17" s="16"/>
       <c r="D17" s="7">
         <v>0.5</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="21"/>
-      <c r="B18" s="17" t="s">
+      <c r="A18" s="23"/>
+      <c r="B18" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="18"/>
+      <c r="C18" s="16"/>
       <c r="D18" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="21"/>
-      <c r="B19" s="17" t="s">
+      <c r="A19" s="23"/>
+      <c r="B19" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C19" s="18"/>
+      <c r="C19" s="16"/>
       <c r="D19" s="8">
         <v>2.5</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="21"/>
-      <c r="B20" s="17" t="s">
+      <c r="A20" s="23"/>
+      <c r="B20" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C20" s="18"/>
+      <c r="C20" s="16"/>
       <c r="D20" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="21"/>
-      <c r="B21" s="49"/>
-      <c r="C21" s="50"/>
+      <c r="A21" s="23"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="20"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="21"/>
-      <c r="B22" s="43"/>
-      <c r="C22" s="44"/>
+      <c r="A22" s="23"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="18"/>
       <c r="D22" s="8"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="21"/>
-      <c r="B23" s="17"/>
-      <c r="C23" s="18"/>
+      <c r="A23" s="23"/>
+      <c r="B23" s="15"/>
+      <c r="C23" s="16"/>
       <c r="D23" s="8"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="21"/>
+      <c r="A24" s="23"/>
       <c r="B24" s="2" t="s">
         <v>6</v>
       </c>
@@ -1497,97 +1576,97 @@
       </c>
     </row>
     <row r="25" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="21"/>
-      <c r="B25" s="22" t="s">
+      <c r="A25" s="23"/>
+      <c r="B25" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="C25" s="23"/>
-      <c r="D25" s="24"/>
+      <c r="C25" s="25"/>
+      <c r="D25" s="26"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="20">
+      <c r="A26" s="22">
         <v>46157</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B26" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C26" s="18"/>
+      <c r="C26" s="16"/>
       <c r="D26" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="17" t="s">
+      <c r="A27" s="23"/>
+      <c r="B27" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C27" s="18"/>
+      <c r="C27" s="16"/>
       <c r="D27" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="21"/>
-      <c r="B28" s="17" t="s">
+      <c r="A28" s="23"/>
+      <c r="B28" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C28" s="18"/>
+      <c r="C28" s="16"/>
       <c r="D28" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="21"/>
-      <c r="B29" s="17" t="s">
+      <c r="A29" s="23"/>
+      <c r="B29" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="C29" s="18"/>
+      <c r="C29" s="16"/>
       <c r="D29" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A30" s="21"/>
-      <c r="B30" s="17" t="s">
+      <c r="A30" s="23"/>
+      <c r="B30" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C30" s="18"/>
+      <c r="C30" s="16"/>
       <c r="D30" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A31" s="21"/>
-      <c r="B31" s="17" t="s">
+      <c r="A31" s="23"/>
+      <c r="B31" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C31" s="18"/>
+      <c r="C31" s="16"/>
       <c r="D31" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A32" s="21"/>
-      <c r="B32" s="17" t="s">
+      <c r="A32" s="23"/>
+      <c r="B32" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C32" s="18"/>
+      <c r="C32" s="16"/>
       <c r="D32" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A33" s="21"/>
-      <c r="B33" s="17" t="s">
+      <c r="A33" s="23"/>
+      <c r="B33" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="C33" s="18"/>
+      <c r="C33" s="16"/>
       <c r="D33" s="8">
         <v>0.3</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A34" s="21"/>
+      <c r="A34" s="23"/>
       <c r="B34" s="47" t="s">
         <v>31</v>
       </c>
@@ -1597,35 +1676,35 @@
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A35" s="21"/>
-      <c r="B35" s="26" t="s">
+      <c r="A35" s="23"/>
+      <c r="B35" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="C35" s="27"/>
+      <c r="C35" s="29"/>
       <c r="D35" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A36" s="21"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="14"/>
+      <c r="A36" s="23"/>
+      <c r="B36" s="30"/>
+      <c r="C36" s="31"/>
       <c r="D36" s="8"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A37" s="21"/>
+      <c r="A37" s="23"/>
       <c r="B37" s="45"/>
       <c r="C37" s="46"/>
       <c r="D37" s="8"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A38" s="21"/>
+      <c r="A38" s="23"/>
       <c r="B38" s="45"/>
       <c r="C38" s="46"/>
       <c r="D38" s="8"/>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A39" s="21"/>
+      <c r="A39" s="23"/>
       <c r="B39" s="2" t="s">
         <v>6</v>
       </c>
@@ -1638,95 +1717,95 @@
       </c>
     </row>
     <row r="40" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="21"/>
-      <c r="B40" s="22" t="s">
+      <c r="A40" s="23"/>
+      <c r="B40" s="24" t="s">
         <v>40</v>
       </c>
-      <c r="C40" s="23"/>
-      <c r="D40" s="24"/>
+      <c r="C40" s="25"/>
+      <c r="D40" s="26"/>
     </row>
     <row r="41" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="20">
+      <c r="A41" s="22">
         <v>46160</v>
       </c>
-      <c r="B41" s="28" t="s">
+      <c r="B41" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="C41" s="29"/>
+      <c r="C41" s="31"/>
       <c r="D41" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A42" s="21"/>
-      <c r="B42" s="17" t="s">
+      <c r="A42" s="23"/>
+      <c r="B42" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="C42" s="18"/>
+      <c r="C42" s="16"/>
       <c r="D42" s="8">
         <v>0.5</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A43" s="21"/>
-      <c r="B43" s="17" t="s">
+      <c r="A43" s="23"/>
+      <c r="B43" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="C43" s="18"/>
+      <c r="C43" s="16"/>
       <c r="D43" s="8">
         <v>1.5</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A44" s="21"/>
-      <c r="B44" s="17" t="s">
+      <c r="A44" s="23"/>
+      <c r="B44" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="C44" s="18"/>
+      <c r="C44" s="16"/>
       <c r="D44" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A45" s="21"/>
-      <c r="B45" s="17" t="s">
+      <c r="A45" s="23"/>
+      <c r="B45" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C45" s="18"/>
+      <c r="C45" s="16"/>
       <c r="D45" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A46" s="21"/>
-      <c r="B46" s="17" t="s">
+      <c r="A46" s="23"/>
+      <c r="B46" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="C46" s="18"/>
+      <c r="C46" s="16"/>
       <c r="D46" s="8">
         <v>2</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A47" s="21"/>
-      <c r="B47" s="17"/>
-      <c r="C47" s="18"/>
+      <c r="A47" s="23"/>
+      <c r="B47" s="15"/>
+      <c r="C47" s="16"/>
       <c r="D47" s="8"/>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="21"/>
-      <c r="B48" s="17"/>
-      <c r="C48" s="18"/>
+      <c r="A48" s="23"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="16"/>
       <c r="D48" s="8"/>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="21"/>
-      <c r="B49" s="15"/>
-      <c r="C49" s="16"/>
+      <c r="A49" s="23"/>
+      <c r="B49" s="13"/>
+      <c r="C49" s="14"/>
       <c r="D49" s="8"/>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="21"/>
+      <c r="A50" s="23"/>
       <c r="B50" s="2" t="s">
         <v>6</v>
       </c>
@@ -1739,55 +1818,59 @@
       </c>
     </row>
     <row r="51" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="25"/>
-      <c r="B51" s="30" t="s">
+      <c r="A51" s="27"/>
+      <c r="B51" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="C51" s="31"/>
-      <c r="D51" s="32"/>
-    </row>
-    <row r="52" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="20">
+      <c r="C51" s="33"/>
+      <c r="D51" s="34"/>
+    </row>
+    <row r="52" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="22">
         <v>46161</v>
       </c>
-      <c r="B52" s="17" t="s">
+      <c r="B52" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="C52" s="18"/>
+      <c r="C52" s="16"/>
       <c r="D52" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A53" s="21"/>
-      <c r="B53" s="17" t="s">
+      <c r="A53" s="23"/>
+      <c r="B53" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C53" s="18"/>
+      <c r="C53" s="16"/>
       <c r="D53" s="8">
         <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A54" s="21"/>
-      <c r="B54" s="17"/>
-      <c r="C54" s="18"/>
-      <c r="D54" s="8"/>
+      <c r="A54" s="23"/>
+      <c r="B54" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C54" s="16"/>
+      <c r="D54" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A55" s="21"/>
-      <c r="B55" s="17"/>
-      <c r="C55" s="18"/>
+      <c r="A55" s="23"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="16"/>
       <c r="D55" s="8"/>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A56" s="21"/>
-      <c r="B56" s="17"/>
-      <c r="C56" s="18"/>
+      <c r="A56" s="23"/>
+      <c r="B56" s="15"/>
+      <c r="C56" s="16"/>
       <c r="D56" s="8"/>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A57" s="21"/>
+      <c r="A57" s="23"/>
       <c r="B57" s="2" t="s">
         <v>6</v>
       </c>
@@ -1800,45 +1883,59 @@
       </c>
     </row>
     <row r="58" spans="1:4" ht="78.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="25"/>
-      <c r="B58" s="30" t="s">
+      <c r="A58" s="27"/>
+      <c r="B58" s="32" t="s">
         <v>41</v>
       </c>
-      <c r="C58" s="31"/>
-      <c r="D58" s="32"/>
+      <c r="C58" s="33"/>
+      <c r="D58" s="34"/>
     </row>
     <row r="59" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="20"/>
-      <c r="B59" s="41"/>
-      <c r="C59" s="42"/>
-      <c r="D59" s="7"/>
+      <c r="A59" s="22">
+        <v>46163</v>
+      </c>
+      <c r="B59" s="28" t="s">
+        <v>44</v>
+      </c>
+      <c r="C59" s="29"/>
+      <c r="D59" s="7">
+        <v>0.1</v>
+      </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A60" s="21"/>
-      <c r="B60" s="17"/>
-      <c r="C60" s="18"/>
-      <c r="D60" s="8"/>
+      <c r="A60" s="23"/>
+      <c r="B60" s="28" t="s">
+        <v>43</v>
+      </c>
+      <c r="C60" s="29"/>
+      <c r="D60" s="8">
+        <v>1.9</v>
+      </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A61" s="21"/>
-      <c r="B61" s="17"/>
-      <c r="C61" s="18"/>
-      <c r="D61" s="8"/>
+      <c r="A61" s="23"/>
+      <c r="B61" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C61" s="16"/>
+      <c r="D61" s="8">
+        <v>2</v>
+      </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A62" s="21"/>
-      <c r="B62" s="17"/>
-      <c r="C62" s="18"/>
+      <c r="A62" s="23"/>
+      <c r="B62" s="15"/>
+      <c r="C62" s="16"/>
       <c r="D62" s="8"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A63" s="21"/>
-      <c r="B63" s="17"/>
-      <c r="C63" s="18"/>
+      <c r="A63" s="23"/>
+      <c r="B63" s="15"/>
+      <c r="C63" s="16"/>
       <c r="D63" s="8"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A64" s="21"/>
+      <c r="A64" s="23"/>
       <c r="B64" s="2" t="s">
         <v>6</v>
       </c>
@@ -1847,47 +1944,49 @@
       </c>
       <c r="D64" s="9">
         <f>SUM(D59:D63)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="65" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="25"/>
-      <c r="B65" s="30"/>
-      <c r="C65" s="31"/>
-      <c r="D65" s="32"/>
-    </row>
-    <row r="66" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="20"/>
-      <c r="B66" s="41"/>
-      <c r="C66" s="42"/>
+      <c r="A65" s="27"/>
+      <c r="B65" s="32" t="s">
+        <v>45</v>
+      </c>
+      <c r="C65" s="33"/>
+      <c r="D65" s="34"/>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A66" s="22"/>
+      <c r="B66" s="43"/>
+      <c r="C66" s="44"/>
       <c r="D66" s="7"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A67" s="21"/>
-      <c r="B67" s="17"/>
-      <c r="C67" s="18"/>
+      <c r="A67" s="23"/>
+      <c r="B67" s="15"/>
+      <c r="C67" s="16"/>
       <c r="D67" s="8"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A68" s="21"/>
-      <c r="B68" s="17"/>
-      <c r="C68" s="18"/>
+      <c r="A68" s="23"/>
+      <c r="B68" s="15"/>
+      <c r="C68" s="16"/>
       <c r="D68" s="8"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A69" s="21"/>
-      <c r="B69" s="17"/>
-      <c r="C69" s="18"/>
+      <c r="A69" s="23"/>
+      <c r="B69" s="15"/>
+      <c r="C69" s="16"/>
       <c r="D69" s="8"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A70" s="21"/>
-      <c r="B70" s="17"/>
-      <c r="C70" s="18"/>
+      <c r="A70" s="23"/>
+      <c r="B70" s="13"/>
+      <c r="C70" s="14"/>
       <c r="D70" s="8"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A71" s="21"/>
+      <c r="A71" s="23"/>
       <c r="B71" s="2" t="s">
         <v>6</v>
       </c>
@@ -1900,43 +1999,43 @@
       </c>
     </row>
     <row r="72" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="25"/>
-      <c r="B72" s="30"/>
-      <c r="C72" s="31"/>
-      <c r="D72" s="32"/>
-    </row>
-    <row r="73" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="20"/>
-      <c r="B73" s="41"/>
-      <c r="C73" s="42"/>
+      <c r="A72" s="27"/>
+      <c r="B72" s="32"/>
+      <c r="C72" s="33"/>
+      <c r="D72" s="34"/>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A73" s="22"/>
+      <c r="B73" s="43"/>
+      <c r="C73" s="44"/>
       <c r="D73" s="7"/>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A74" s="21"/>
-      <c r="B74" s="17"/>
-      <c r="C74" s="18"/>
+      <c r="A74" s="23"/>
+      <c r="B74" s="15"/>
+      <c r="C74" s="16"/>
       <c r="D74" s="8"/>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A75" s="21"/>
-      <c r="B75" s="17"/>
-      <c r="C75" s="18"/>
+      <c r="A75" s="23"/>
+      <c r="B75" s="15"/>
+      <c r="C75" s="16"/>
       <c r="D75" s="8"/>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A76" s="21"/>
-      <c r="B76" s="17"/>
-      <c r="C76" s="18"/>
+      <c r="A76" s="23"/>
+      <c r="B76" s="15"/>
+      <c r="C76" s="16"/>
       <c r="D76" s="8"/>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A77" s="21"/>
-      <c r="B77" s="17"/>
-      <c r="C77" s="18"/>
+      <c r="A77" s="23"/>
+      <c r="B77" s="13"/>
+      <c r="C77" s="14"/>
       <c r="D77" s="8"/>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A78" s="21"/>
+      <c r="A78" s="23"/>
       <c r="B78" s="2" t="s">
         <v>6</v>
       </c>
@@ -1949,43 +2048,43 @@
       </c>
     </row>
     <row r="79" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="25"/>
-      <c r="B79" s="30"/>
-      <c r="C79" s="31"/>
-      <c r="D79" s="32"/>
+      <c r="A79" s="27"/>
+      <c r="B79" s="32"/>
+      <c r="C79" s="33"/>
+      <c r="D79" s="34"/>
     </row>
     <row r="80" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="20"/>
-      <c r="B80" s="41"/>
-      <c r="C80" s="42"/>
+      <c r="A80" s="22"/>
+      <c r="B80" s="43"/>
+      <c r="C80" s="44"/>
       <c r="D80" s="7"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A81" s="21"/>
-      <c r="B81" s="17"/>
-      <c r="C81" s="18"/>
+      <c r="A81" s="23"/>
+      <c r="B81" s="15"/>
+      <c r="C81" s="16"/>
       <c r="D81" s="8"/>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A82" s="21"/>
-      <c r="B82" s="17"/>
-      <c r="C82" s="18"/>
+      <c r="A82" s="23"/>
+      <c r="B82" s="15"/>
+      <c r="C82" s="16"/>
       <c r="D82" s="8"/>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A83" s="21"/>
-      <c r="B83" s="17"/>
-      <c r="C83" s="18"/>
+      <c r="A83" s="23"/>
+      <c r="B83" s="15"/>
+      <c r="C83" s="16"/>
       <c r="D83" s="8"/>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A84" s="21"/>
-      <c r="B84" s="17"/>
-      <c r="C84" s="18"/>
+      <c r="A84" s="23"/>
+      <c r="B84" s="15"/>
+      <c r="C84" s="16"/>
       <c r="D84" s="8"/>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A85" s="21"/>
+      <c r="A85" s="23"/>
       <c r="B85" s="2" t="s">
         <v>6</v>
       </c>
@@ -1998,43 +2097,43 @@
       </c>
     </row>
     <row r="86" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="21"/>
-      <c r="B86" s="22"/>
-      <c r="C86" s="23"/>
-      <c r="D86" s="24"/>
+      <c r="A86" s="23"/>
+      <c r="B86" s="24"/>
+      <c r="C86" s="25"/>
+      <c r="D86" s="26"/>
     </row>
     <row r="87" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="20"/>
-      <c r="B87" s="41"/>
-      <c r="C87" s="42"/>
+      <c r="A87" s="22"/>
+      <c r="B87" s="43"/>
+      <c r="C87" s="44"/>
       <c r="D87" s="7"/>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A88" s="21"/>
-      <c r="B88" s="17"/>
-      <c r="C88" s="18"/>
+      <c r="A88" s="23"/>
+      <c r="B88" s="15"/>
+      <c r="C88" s="16"/>
       <c r="D88" s="8"/>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A89" s="21"/>
-      <c r="B89" s="17"/>
-      <c r="C89" s="18"/>
+      <c r="A89" s="23"/>
+      <c r="B89" s="15"/>
+      <c r="C89" s="16"/>
       <c r="D89" s="8"/>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A90" s="21"/>
-      <c r="B90" s="17"/>
-      <c r="C90" s="18"/>
+      <c r="A90" s="23"/>
+      <c r="B90" s="15"/>
+      <c r="C90" s="16"/>
       <c r="D90" s="8"/>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A91" s="21"/>
-      <c r="B91" s="17"/>
-      <c r="C91" s="18"/>
+      <c r="A91" s="23"/>
+      <c r="B91" s="15"/>
+      <c r="C91" s="16"/>
       <c r="D91" s="8"/>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A92" s="21"/>
+      <c r="A92" s="23"/>
       <c r="B92" s="2" t="s">
         <v>6</v>
       </c>
@@ -2047,43 +2146,43 @@
       </c>
     </row>
     <row r="93" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="25"/>
-      <c r="B93" s="30"/>
-      <c r="C93" s="31"/>
-      <c r="D93" s="32"/>
+      <c r="A93" s="27"/>
+      <c r="B93" s="32"/>
+      <c r="C93" s="33"/>
+      <c r="D93" s="34"/>
     </row>
     <row r="94" spans="1:4" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="20"/>
-      <c r="B94" s="41"/>
-      <c r="C94" s="42"/>
+      <c r="A94" s="22"/>
+      <c r="B94" s="43"/>
+      <c r="C94" s="44"/>
       <c r="D94" s="7"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A95" s="21"/>
-      <c r="B95" s="17"/>
-      <c r="C95" s="18"/>
+      <c r="A95" s="23"/>
+      <c r="B95" s="15"/>
+      <c r="C95" s="16"/>
       <c r="D95" s="8"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A96" s="21"/>
-      <c r="B96" s="17"/>
-      <c r="C96" s="18"/>
+      <c r="A96" s="23"/>
+      <c r="B96" s="15"/>
+      <c r="C96" s="16"/>
       <c r="D96" s="8"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A97" s="21"/>
-      <c r="B97" s="17"/>
-      <c r="C97" s="18"/>
+      <c r="A97" s="23"/>
+      <c r="B97" s="15"/>
+      <c r="C97" s="16"/>
       <c r="D97" s="8"/>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A98" s="21"/>
-      <c r="B98" s="17"/>
-      <c r="C98" s="18"/>
+      <c r="A98" s="23"/>
+      <c r="B98" s="15"/>
+      <c r="C98" s="16"/>
       <c r="D98" s="8"/>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A99" s="21"/>
+      <c r="A99" s="23"/>
       <c r="B99" s="2" t="s">
         <v>6</v>
       </c>
@@ -2096,10 +2195,10 @@
       </c>
     </row>
     <row r="100" spans="1:4" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="25"/>
-      <c r="B100" s="30"/>
-      <c r="C100" s="31"/>
-      <c r="D100" s="32"/>
+      <c r="A100" s="27"/>
+      <c r="B100" s="32"/>
+      <c r="C100" s="33"/>
+      <c r="D100" s="34"/>
     </row>
     <row r="101" spans="1:4" ht="12" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="11"/>
@@ -2109,19 +2208,19 @@
       </c>
       <c r="D101" s="12">
         <f>D15+D24+D39+D50+D57+D64+D71+D78+D85+D92+D99</f>
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A102" s="19" t="s">
+      <c r="A102" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B102" s="19"/>
-      <c r="C102" s="19"/>
-      <c r="D102" s="19"/>
+      <c r="B102" s="21"/>
+      <c r="C102" s="21"/>
+      <c r="D102" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="99">
+  <mergeCells count="100">
     <mergeCell ref="A26:A40"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
@@ -2134,6 +2233,7 @@
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B36:C36"/>
     <mergeCell ref="B72:D72"/>
     <mergeCell ref="A73:A79"/>
     <mergeCell ref="B73:C73"/>
@@ -2223,84 +2323,84 @@
     <mergeCell ref="B47:C47"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:D15 D17:D20 D22:D24 D26">
-    <cfRule type="containsText" dxfId="19" priority="24" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="23" priority="24" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D26 D6:D15 D17:D20 D22:D24">
-    <cfRule type="containsText" dxfId="18" priority="23" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="22" priority="23" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D6)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D26:D39 D41:D50">
-    <cfRule type="containsText" dxfId="17" priority="3" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="21" priority="3" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D26)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="4" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="20" priority="4" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D26)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D52:D57">
-    <cfRule type="containsText" dxfId="15" priority="17" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="19" priority="17" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D52)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="14" priority="18" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="18" priority="18" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D52)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D59:D64">
-    <cfRule type="containsText" dxfId="13" priority="9" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="17" priority="9" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D59)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="12" priority="10" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="16" priority="10" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D59)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D66:D71">
-    <cfRule type="containsText" dxfId="11" priority="7" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="15" priority="7" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D66)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="10" priority="8" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="14" priority="8" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D66)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D73:D78">
-    <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="13" priority="5" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D73)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="12" priority="6" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D73)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D80:D85">
-    <cfRule type="containsText" dxfId="7" priority="15" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="11" priority="15" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D80)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="16" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="10" priority="16" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D80)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D87:D92">
-    <cfRule type="containsText" dxfId="5" priority="13" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="9" priority="13" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D87)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="14" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="8" priority="14" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D87)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D94:D99">
-    <cfRule type="containsText" dxfId="3" priority="11" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="7" priority="11" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D94)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="12" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="6" priority="12" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D94)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D101">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Terminé">
+    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="Terminé">
       <formula>NOT(ISERROR(SEARCH("Terminé",D101)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="2" operator="containsText" text="En cours">
+    <cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="En cours">
       <formula>NOT(ISERROR(SEARCH("En cours",D101)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>